<commit_message>
Einrichtblatt (Test): jedes Werkzeugfeld gleich, A4 quer, ohne Autom.-Nr. und FA Nr.
Alle Reihen gleich hoch, Kopf je Typ, darunter Platz für Bemerkungen.
Excel einlesen erkennt das Mass auch nach einer Leerzeile.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015CEWSjPmHA2CFkwJ2RMC2A
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-app-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-app-beispiel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>Werkzeug- Protokoll-SR32J</t>
   </si>
@@ -25,6 +25,9 @@
     <t>T3100</t>
   </si>
   <si>
+    <t>T400</t>
+  </si>
+  <si>
     <t>Abstechen</t>
   </si>
   <si>
@@ -40,6 +43,9 @@
     <t>M5</t>
   </si>
   <si>
+    <t>Ø 3.50</t>
+  </si>
+  <si>
     <t>Vischer &amp; Bolli AG</t>
   </si>
   <si>
@@ -53,6 +59,9 @@
   </si>
   <si>
     <t>Former M5</t>
+  </si>
+  <si>
+    <t>HYP-HP-3D Ø3.50</t>
   </si>
   <si>
     <t>Programm Path 1:</t>
@@ -501,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -509,7 +518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -518,6 +527,9 @@
       </c>
       <c r="E3" t="s">
         <v>3</v>
+      </c>
+      <c r="G3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -525,138 +537,154 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
         <v>12</v>
       </c>
-      <c r="E9" t="s">
-        <v>13</v>
+    </row>
+    <row r="10" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>